<commit_message>
Cut the first order to one cubic metre and a check under 1 million.
The previous draft was 2.3 m3 and 1.76 million. This one is 0.81 m3, 4095 EUR, and 737 thousand rubles all-in, still in profit after VAT and profit tax.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -985,7 +985,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Просим подтвердить, что эти нетто ещё действуют, и написать, какая скидка возможна по дилерской схеме. Количество — наш черновик первого заказа, не заявка. FLY в инвойсе есть, в первый заказ не берём.</t>
+          <t>Просим подтвердить, что эти нетто ещё действуют, и написать, какая скидка возможна по дилерской схеме. Количество — черновик первого заказа на один куб, не заявка. BLASTER и FLY в инвойсе есть, в этот куб не берём.</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
         <v>46</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E5" s="8">
         <f>C5*D5</f>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Самая сильная экономика среди редукторов</t>
+          <t>В первый куб, около 20 шт</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E6" s="8">
         <f>C6*D6</f>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>До ~250 л.с.</t>
+          <t>В первый куб, около 20 шт</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8">
         <f>C7*D7</f>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Самый частый редуктор, до ~170 л.с.</t>
+          <t>В первый куб, около 20 шт</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
         <v>4.5</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="E8" s="8">
         <f>C8*D8</f>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Основной фильтр в заказе</t>
+          <t>Основной фильтр в кубе, около 400 шт</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
         <v>3.5</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8">
         <f>C9*D9</f>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Второй фильтр, штук меньше</t>
+          <t>В инвойсе есть. В этот куб не берём</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
         <v>0.7</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="E10" s="8">
         <f>C10*D10</f>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Ходовой расходник</t>
+          <t>Ходовой расходник, около 250 шт</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>В инвойсе есть. В первый заказ не берём</t>
+          <t>В инвойсе есть. В этот куб не берём</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch the first order to 130 AT13 reducers, the highest profit under 1 million.
A mixed cube left about 59 thousand after tax. Filling the cash cap with AT13 XP lands at 984 thousand in and 147 thousand net, and any other SKU in the same budget earns less.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -985,7 +985,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Просим подтвердить, что эти нетто ещё действуют, и написать, какая скидка возможна по дилерской схеме. Количество — черновик первого заказа на один куб, не заявка. BLASTER и FLY в инвойсе есть, в этот куб не берём.</t>
+          <t>Первый заказ смотрим как 130 шт AT13 XP. Остальное из инвойса в этот заход не берём. Просим подтвердить 46 € и написать скидку по дилерской схеме. Количество — черновик, не заявка.</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
         <v>46</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="E5" s="8">
         <f>C5*D5</f>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>В первый куб, около 20 шт</t>
+          <t>Первый заказ, около 130 шт</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8">
         <f>C6*D6</f>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>В первый куб, около 20 шт</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
         <v>26</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8">
         <f>C7*D7</f>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>В первый куб, около 20 шт</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
         <v>4.5</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8">
         <f>C8*D8</f>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Основной фильтр в кубе, около 400 шт</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>В инвойсе есть. В этот куб не берём</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
         <v>0.7</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="E10" s="8">
         <f>C10*D10</f>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Ходовой расходник, около 250 шт</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>В инвойсе есть. В этот куб не берём</t>
+          <t>В инвойсе есть. В этот заказ не берём</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop profit tax and price two orders: 130 AT13, or a full cubic metre.
European invoices stay netto. Russian import VAT stays in the check. On that model 130 AT13 returns 264 thousand, and the five-line cube returns 202 thousand, both under 1 million.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Нет вашей цены" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Уже есть в инвойсе" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Два черновика заказа" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Нет вашей цены'!$A$4:$F$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Нет вашей цены'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Уже есть в инвойсе'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Два черновика заказа'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="# ##0"/>
     <numFmt numFmtId="165" formatCode="# ##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,11 +53,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -100,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -115,18 +110,9 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,10 +496,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Это не анкета и заполнять её не нужно. Удобнее прислать ваш полный прайс или типовой инвойс: нетто в евро, наличие, срок. Мы сами сопоставим. Полкой Digitronic ниже указана розница в России, это не ваша цена.</t>
+          <t>Это не анкета, заполнять её не нужно. Удобнее прислать полный прайс: нетто в евро, наличие, срок. Полка Digitronic — розница в России, не ваша цена.</t>
         </is>
       </c>
     </row>
@@ -635,7 +621,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Дороже обычного MP48, в наличии</t>
+          <t>Дороже обычного MP48</t>
         </is>
       </c>
     </row>
@@ -947,14 +933,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LГБО · позиции без вашей цены</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -964,58 +942,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Позиции, цена которых у нас уже есть</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+          <t>Два черновика первого заказа. Это альтернативы, количества не складывать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Первый заказ смотрим как 130 шт AT13 XP. Остальное из инвойса в этот заход не берём. Просим подтвердить 46 € и написать скидку по дилерской схеме. Количество — черновик, не заявка.</t>
+          <t>Просим подтвердить нетто из инвойса и написать возможную дилерскую скидку. Количество — ориентир, не заявка.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>Вариант</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Название</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Артикул</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Цена в инвойсе, €</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Смотрим в первый заказ, шт</t>
-        </is>
-      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Сумма по инвойсу, €</t>
+          <t>Штук</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Сумма, €</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -1024,216 +1008,268 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Один артикул</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
           <t>AT13 XP</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>RGDG3990</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="D5" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="E5" s="5" t="n">
         <v>130</v>
       </c>
-      <c r="E5" s="8">
-        <f>C5*D5</f>
+      <c r="F5" s="6">
+        <f>D5*E5</f>
         <v/>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Первый заказ, около 130 шт</t>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Основной вариант</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>AT09 Nordic XP</t>
+          <t>Комплект на куб</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>RGDG3895</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8">
-        <f>C6*D6</f>
+          <t>BLASTER Y 12×2/12</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>BLASTER Y 12x2/12</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="F6" s="6">
+        <f>D6*E6</f>
         <v/>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Фильтр</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>AT09 Nordic</t>
+          <t>Комплект на куб</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>RGDG3890</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8">
-        <f>C7*D7</f>
+          <t>FLS 12×12</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>FL01S 12/12</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="F7" s="6">
+        <f>D7*E7</f>
         <v/>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Фильтр</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>BLASTER Y 12×2/12</t>
+          <t>Комплект на куб</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>BLASTER Y 12x2/12</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="8">
-        <f>C8*D8</f>
+          <t>AT09 Nordic</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>RGDG3890</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" s="6">
+        <f>D8*E8</f>
         <v/>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Редуктор</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>BLASTER 12×12</t>
+          <t>Комплект на куб</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>BLASTER 12х12</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="8">
-        <f>C9*D9</f>
+          <t>AT09 Nordic XP</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>RGDG3895</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="6">
+        <f>D9*E9</f>
         <v/>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Редуктор</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>FLS 12×12</t>
+          <t>Комплект на куб</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>FL01S 12/12</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="8">
-        <f>C10*D10</f>
+          <t>AT13 XP</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>RGDG3990</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" s="6">
+        <f>D10*E10</f>
         <v/>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Редуктор</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Не берём</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>BLASTER 12×12</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>BLASTER 12х12</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="6">
+        <f>D11*E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>В инвойсе есть, в эти черновики не входит</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Не берём</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>FLY 12 / 2×12</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>FL01Y 12/12</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="8">
-        <f>C11*D11</f>
+      <c r="F12" s="6">
+        <f>D12*E12</f>
         <v/>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть. В этот заказ не берём</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Итого в черновике</t>
-        </is>
-      </c>
-      <c r="D12" s="10">
-        <f>SUM(D5:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="11">
-        <f>SUM(E5:E11)</f>
-        <v/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>В инвойсе есть, в эти черновики не входит</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;LГБО · черновик первого заказа</oddHeader>
+    <oddHeader>&amp;LГБО · черновики первого заказа</oddHeader>
     <oddFooter/>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
Rewrite the supplier note and Excel as an export enquiry in euros.
The file she can forward no longer mentions Kazan, rubles, customs, or a budget. Prices stay in euros, with zloty only if that is how they quote.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -7,13 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Нет вашей цены" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Два черновика заказа" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Нет в инвойсе" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Составы в евро" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Нет вашей цены'!$A$4:$F$17</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Нет вашей цены'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Два черновика заказа'!$1:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Нет в инвойсе'!$A$4:$D$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Нет в инвойсе'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Составы в евро'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,8 +107,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -478,28 +481,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Позиции, по которым у нас нет вашей цены</t>
+          <t>Артикулы, которых не было в прошлом инвойсе</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Это не анкета, заполнять её не нужно. Удобнее прислать полный прайс: нетто в евро, наличие, срок. Полка Digitronic — розница в России, не ваша цена.</t>
+          <t>Это не анкета. Удобнее прислать полный прайс: нетто в евро или в злотых, наличие и срок. Мы сами сопоставим.</t>
         </is>
       </c>
     </row>
@@ -521,17 +522,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Полка Digitronic, ₽</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Наличие у Digitronic</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Зачем смотрим</t>
+          <t>Что хотим увидеть в прайсе</t>
         </is>
       </c>
     </row>
@@ -551,17 +542,9 @@
           <t>616000573</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
-        <v>13200</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Ходовой комплект 4 цил.</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -581,17 +564,9 @@
           <t>616000087</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>15600</v>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Ходовой комплект 4 цил.</t>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -611,17 +586,9 @@
           <t>616000089</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>18200</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Дороже обычного MP48</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -641,17 +608,9 @@
           <t>WEG-AMD024409999-000</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>13300</v>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>На российской полке нет в наличии</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -671,17 +630,9 @@
           <t>WEG-AMD028409999-300</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>23500</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>На российской полке нет в наличии</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -701,17 +652,9 @@
           <t>WEG-AMD030609999-300</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>23300</v>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>На российской полке нет в наличии</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -731,17 +674,9 @@
           <t>WEG-AMD030809999-300</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>28000</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>На российской полке нет в наличии</t>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -761,17 +696,9 @@
           <t>MVDG0205.1</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
-        <v>5550</v>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Класс A</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -791,17 +718,9 @@
           <t>MVDG0012</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>4150</v>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>С заправочным устройством</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -821,17 +740,9 @@
           <t>620500170</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Форсуночная рейка</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -851,17 +762,9 @@
           <t>33.EVG.13</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>5550</v>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Форсуночная рейка</t>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -881,17 +784,9 @@
           <t>TP6-48</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
-        <v>11300</v>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Термопластик</t>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
@@ -911,25 +806,17 @@
           <t>ТР8-48</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n">
-        <v>13900</v>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>много</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Термопластик</t>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>нетто, наличие, срок</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F17"/>
+  <autoFilter ref="A4:D17"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -942,36 +829,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Два черновика первого заказа. Это альтернативы, количества не складывать.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
+          <t>Два состава по прошлому инвойсу. Это альтернативы, количества не складывать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Просим подтвердить нетто из инвойса и написать возможную дилерскую скидку. Количество — ориентир, не заявка.</t>
+          <t>Просим подтвердить нетто в евро и написать, какая индивидуальная цена возможна. Если у вас прайс в злотых, можно прислать в злотых. Количество — ориентир, не заявка.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Вариант</t>
+          <t>Состав</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -997,18 +883,13 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Сумма, €</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Комментарий</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Один артикул</t>
+          <t>Первый</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1024,23 +905,18 @@
       <c r="D5" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>130</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Основной вариант</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Комплект на куб</t>
+          <t>Второй, комплект</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1053,26 +929,21 @@
           <t>BLASTER Y 12x2/12</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>4.5</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="7">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Фильтр</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Комплект на куб</t>
+          <t>Второй, комплект</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1085,26 +956,21 @@
           <t>FL01S 12/12</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Фильтр</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Комплект на куб</t>
+          <t>Второй, комплект</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1120,23 +986,18 @@
       <c r="D8" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Редуктор</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Комплект на куб</t>
+          <t>Второй, комплект</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1152,23 +1013,18 @@
       <c r="D9" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="7">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Редуктор</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Комплект на куб</t>
+          <t>Второй, комплект</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1184,97 +1040,20 @@
       <c r="D10" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="7">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Редуктор</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Не берём</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>BLASTER 12×12</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>BLASTER 12х12</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6">
-        <f>D11*E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть, в эти черновики не входит</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Не берём</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>FLY 12 / 2×12</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>FL01Y 12/12</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <f>D12*E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>В инвойсе есть, в эти черновики не входит</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LГБО · черновики первого заказа</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rewrite the supplier note as a follow-up, not a new introduction.
She already sent an invoice and the thread stopped. The message now picks that up: two order options, a request for the missing prices or the full list, and individual terms.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -493,14 +493,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Артикулы, которых не было в прошлом инвойсе</t>
+          <t>Чего не было в инвойсе</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Это не анкета. Удобнее прислать полный прайс: нетто в евро или в злотых, наличие и срок. Мы сами сопоставим.</t>
+          <t>Заполнять не нужно. Проще прислать весь перечень: нетто в евро или в злотых, наличие и срок.</t>
         </is>
       </c>
     </row>
@@ -843,14 +843,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Два состава по прошлому инвойсу. Это альтернативы, количества не складывать.</t>
+          <t>Два варианта первого заказа. Это на выбор, не вместе.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Просим подтвердить нетто в евро и написать, какая индивидуальная цена возможна. Если у вас прайс в злотых, можно прислать в злотых. Количество — ориентир, не заявка.</t>
+          <t>Цены как в вашем инвойсе, в евро. Напишите, пожалуйста, какая индивидуальная цена возможна. Если прайс в злотых, можно в злотых.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start the supplier note from the order, not from the old invoice.
No thanks for the invoice and no apology for the gap. The note asks which mix to take, for the missing prices or the full list, and for individual terms.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -493,7 +493,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Чего не было в инвойсе</t>
+          <t>Позиции, по которым нужна цена</t>
         </is>
       </c>
     </row>
@@ -843,14 +843,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Два варианта первого заказа. Это на выбор, не вместе.</t>
+          <t>Два варианта заказа. На выбор, не вместе.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Цены как в вашем инвойсе, в евро. Напишите, пожалуйста, какая индивидуальная цена возможна. Если прайс в злотых, можно в злотых.</t>
+          <t>Цены в евро, как они у нас есть. Напишите, какая индивидуальная цена возможна. Если прайс в злотых, можно в злотых.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill Digitronic quote quantities for a ~1M RUB trial and draft Katerina reply.
Excel now has qty on both sheets; reply text states two order options (~5.5–6k EUR goods) and asks for individual net terms.

Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="# ##0"/>
     <numFmt numFmtId="165" formatCode="# ##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,9 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -95,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -116,6 +119,7 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,13 +485,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +505,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Заполнять не нужно. Проще прислать весь перечень: нетто в евро или в злотых, наличие и срок.</t>
+          <t>Кол-во — ориентир на первый пробный заказ (~5,5–6 тыс. € товар / до ~1 млн ₽ с доставкой и таможней). Точный состав по этим позициям — после ваших нетто. Можно прислать весь свой перечень.</t>
         </is>
       </c>
     </row>
@@ -525,6 +530,11 @@
           <t>Что хотим увидеть в прайсе</t>
         </is>
       </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Кол-во, шт (ориентир 1-й заказ)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -547,6 +557,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -569,6 +582,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -591,6 +607,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -613,6 +632,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -635,6 +657,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -657,6 +682,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -679,6 +707,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -701,6 +732,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E12" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -723,6 +757,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -745,6 +782,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E14" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -767,6 +807,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -789,6 +832,9 @@
           <t>нетто, наличие, срок</t>
         </is>
       </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -810,6 +856,9 @@
         <is>
           <t>нетто, наличие, срок</t>
         </is>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -843,14 +892,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Два варианта заказа. На выбор, не вместе.</t>
+          <t>Два варианта первого пробного заказа. На выбор, не вместе. Товар ~5,4–6,0 тыс. € (наш чек с логистикой/таможней до ~1 млн ₽).</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Цены в евро, как они у нас есть. Напишите, какая индивидуальная цена возможна. Если прайс в злотых, можно в злотых.</t>
+          <t>Кол-ва заполнены. Нужна ваша индивидуальная цена нетто EUR (или PLN) и условие скидки от суммы/количества.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite Katerina reply in plain language; drop internal RUB/logistics from the email and Excel notes.
Co-authored-by: GithubRavilS <GithubRavilS@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/zapros-assortiment.xlsx
+++ b/zapros-assortiment.xlsx
@@ -505,7 +505,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Кол-во — ориентир на первый пробный заказ (~5,5–6 тыс. € товар / до ~1 млн ₽ с доставкой и таможней). Точный состав по этим позициям — после ваших нетто. Можно прислать весь свой перечень.</t>
+          <t>Кол-во — ориентир на первый пробный заказ (~5–6 тыс. € по товару). Точный состав по этим позициям — после ваших нетто. Можно прислать весь свой перечень.</t>
         </is>
       </c>
     </row>
@@ -892,14 +892,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Два варианта первого пробного заказа. На выбор, не вместе. Товар ~5,4–6,0 тыс. € (наш чек с логистикой/таможней до ~1 млн ₽).</t>
+          <t>Два варианта первого пробного заказа. На выбор, не вместе. Ориентир ~5–6 тыс. € по товару.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Кол-ва заполнены. Нужна ваша индивидуальная цена нетто EUR (или PLN) и условие скидки от суммы/количества.</t>
+          <t>Кол-ва заполнены. Нужна цена нетто EUR или PLN, наличие, срок и ваши условия на такой объём.</t>
         </is>
       </c>
     </row>

</xml_diff>